<commit_message>
update all supplementary materials and tables
</commit_message>
<xml_diff>
--- a/library_survey_supplementary_materials/supp_table_1a_jacquere_cfd_score_by_alignment_bin.xlsx
+++ b/library_survey_supplementary_materials/supp_table_1a_jacquere_cfd_score_by_alignment_bin.xlsx
@@ -386,7 +386,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>51774</v>
+        <v>48999</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -397,7 +397,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>4101</v>
+        <v>3789</v>
       </c>
       <c r="C3" t="n">
         <v>0.6</v>
@@ -408,7 +408,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>922</v>
+        <v>837</v>
       </c>
       <c r="C4" t="n">
         <v>0.666666667</v>
@@ -419,7 +419,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>330</v>
+        <v>282</v>
       </c>
       <c r="C5" t="n">
         <v>0.666666667</v>
@@ -430,10 +430,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>180</v>
+        <v>152</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6449579835</v>
+        <v>0.648529412</v>
       </c>
     </row>
     <row r="7">
@@ -441,10 +441,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="C7" t="n">
-        <v>0.625</v>
+        <v>0.6449579835</v>
       </c>
     </row>
     <row r="8">
@@ -452,10 +452,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>164</v>
+        <v>121</v>
       </c>
       <c r="C8" t="n">
-        <v>0.4</v>
+        <v>0.454545455</v>
       </c>
     </row>
   </sheetData>

</xml_diff>